<commit_message>
Feat: Comprobantes muestra vendedor y metodo de pago - Reportes muestra resumen total y desglose por pago
</commit_message>
<xml_diff>
--- a/Productos.xlsx
+++ b/Productos.xlsx
@@ -5,16 +5,19 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cupej\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Sistema de Almacen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{59B91E41-A0D3-48BF-88C4-7FDC2DC3C1D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D234472-15CD-4DAB-B066-F4E6EDE99AF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13550" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{F46408A6-377F-47AC-B5A1-E0E7E9D70AB7}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{F46408A6-377F-47AC-B5A1-E0E7E9D70AB7}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$O$279</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -1597,7 +1600,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1607,6 +1610,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1623,9 +1632,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1942,6 +1952,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8AEA3F82-E716-41DC-85DB-78E23D5D9337}">
   <dimension ref="A1:O279"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="30.140625" customWidth="1"/>
+    <col min="2" max="2" width="20.28515625" customWidth="1"/>
+    <col min="4" max="4" width="29.5703125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -5408,25 +5423,27 @@
       </c>
     </row>
     <row r="98" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A98" t="s">
+      <c r="A98" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="B98" t="s">
+      <c r="B98" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="C98" t="s">
+      <c r="C98" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D98" t="s">
-        <v>19</v>
-      </c>
-      <c r="E98" t="s">
-        <v>24</v>
-      </c>
-      <c r="F98" t="s">
+      <c r="D98" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E98" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F98" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="I98">
+      <c r="G98" s="2"/>
+      <c r="H98" s="2"/>
+      <c r="I98" s="2">
         <v>120</v>
       </c>
       <c r="J98">
@@ -10613,6 +10630,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:O279" xr:uid="{8AEA3F82-E716-41DC-85DB-78E23D5D9337}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>